<commit_message>
Unify the website, browser workspace, and document showcase
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/excel/report-workflow.xlsx
+++ b/Website/static/downloads/showcase/excel/report-workflow.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" r:id="R8c27ac53b5a64ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" r:id="R538834cffde745bc"/>
   </x:sheets>
   <x:pivotCaches>
-    <x:pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="R38fb6c1557e0437c"/>
+    <x:pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="R2b79563c32b546ab"/>
   </x:pivotCaches>
 </x:workbook>
 </file>
@@ -289,7 +289,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7811ac066cd34430"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra8d530e277644bd4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -668,7 +668,7 @@
       </c>
     </row>
   </sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="Rd0cd8b71025c41c6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="R221505681ff449ca"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Unify website navigation, browser tools, and document examples (#2462)
* Unify the website, browser workspace, and document showcase

* Run website presentation checks after API generation

* Validate the site logo as the Home navigation link

* Align browser checks and page audits with the shared website
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/excel/report-workflow.xlsx
+++ b/Website/static/downloads/showcase/excel/report-workflow.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" r:id="R8c27ac53b5a64ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" r:id="R538834cffde745bc"/>
   </x:sheets>
   <x:pivotCaches>
-    <x:pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="R38fb6c1557e0437c"/>
+    <x:pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="R2b79563c32b546ab"/>
   </x:pivotCaches>
 </x:workbook>
 </file>
@@ -289,7 +289,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7811ac066cd34430"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra8d530e277644bd4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -668,7 +668,7 @@
       </c>
     </row>
   </sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="Rd0cd8b71025c41c6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="R221505681ff449ca"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>